<commit_message>
Add 23 blocks, update importer
Automated migration updates generated by Experience Modernization Agent.

Changed files: 153
</commit_message>
<xml_diff>
--- a/tools/importer/reports/import-home.report.xlsx
+++ b/tools/importer/reports/import-home.report.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="16" uniqueCount="16">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="117" uniqueCount="88">
   <si>
     <t>_reportFile</t>
   </si>
@@ -19,6 +19,9 @@
     <t>blocks</t>
   </si>
   <si>
+    <t>fragments</t>
+  </si>
+  <si>
     <t>path</t>
   </si>
   <si>
@@ -37,6 +40,51 @@
     <t>url</t>
   </si>
   <si>
+    <t>cancer.report.json</t>
+  </si>
+  <si>
+    <t>["hero-page","cards-carousel","columns-media","columns-media","columns-media","columns-media","hero-article","accordion-faq","search-prompt"]</t>
+  </si>
+  <si>
+    <t/>
+  </si>
+  <si>
+    <t>cancer</t>
+  </si>
+  <si>
+    <t>success</t>
+  </si>
+  <si>
+    <t>content-page</t>
+  </si>
+  <si>
+    <t>2026-10-13T16:51:30.271Z</t>
+  </si>
+  <si>
+    <t>Cancer Overview &amp; Educational Resources | PfizerForAll™</t>
+  </si>
+  <si>
+    <t>https://www.pfizerforall.com/cancer</t>
+  </si>
+  <si>
+    <t>education.report.json</t>
+  </si>
+  <si>
+    <t>["hero-page","carousel-condition","cards-feed","cards-action","banner-cta"]</t>
+  </si>
+  <si>
+    <t>education</t>
+  </si>
+  <si>
+    <t>2026-10-13T16:51:37.277Z</t>
+  </si>
+  <si>
+    <t>Knowledge Hub | PfizerForAll™</t>
+  </si>
+  <si>
+    <t>https://www.pfizerforall.com/education/</t>
+  </si>
+  <si>
     <t>index.report.json</t>
   </si>
   <si>
@@ -46,19 +94,187 @@
     <t>index</t>
   </si>
   <si>
-    <t>success</t>
-  </si>
-  <si>
     <t>home</t>
   </si>
   <si>
-    <t>2026-10-12T22:02:21.770Z</t>
+    <t>2026-10-13T18:40:54.342Z</t>
   </si>
   <si>
     <t>PfizerForAll™ | Official Site</t>
   </si>
   <si>
     <t>https://www.pfizerforall.com/</t>
+  </si>
+  <si>
+    <t>vaccines.report.json</t>
+  </si>
+  <si>
+    <t>["hero-page","cards-article","columns-media","columns-media","banner-cta","cards-nav","quiz-choice","columns-article","quiz-truefalse","form-signup","accordion-faq","search-prompt"]</t>
+  </si>
+  <si>
+    <t>vaccines</t>
+  </si>
+  <si>
+    <t>2026-10-13T16:51:16.362Z</t>
+  </si>
+  <si>
+    <t>Explore Vaccine Options, Eligibility &amp; More | PfizerForAll™</t>
+  </si>
+  <si>
+    <t>https://www.pfizerforall.com/vaccines/</t>
+  </si>
+  <si>
+    <t>find-care/biomarker-testing.report.json</t>
+  </si>
+  <si>
+    <t>["hero-page","cards-article","columns-media","columns-media","cards-nav","quiz-truefalse","accordion-faq","quiz-entry","cards-fact","quote-photo"]</t>
+  </si>
+  <si>
+    <t>find-care/biomarker-testing</t>
+  </si>
+  <si>
+    <t>2026-10-13T16:50:53.746Z</t>
+  </si>
+  <si>
+    <t>Biomarker Testing | Find Care| PfizerForAll™</t>
+  </si>
+  <si>
+    <t>https://www.pfizerforall.com/find-care/biomarker-testing/</t>
+  </si>
+  <si>
+    <t>find-care/cancer-screening.report.json</t>
+  </si>
+  <si>
+    <t>["hero-quiz","cards-icon","columns-callout","cards-carousel","accordion-faq"]</t>
+  </si>
+  <si>
+    <t>/fragments/find-care/cancer-screening/schedule-breast-screening, /fragments/find-care/cancer-screening/schedule-cervical-screening</t>
+  </si>
+  <si>
+    <t>find-care/cancer-screening</t>
+  </si>
+  <si>
+    <t>cancer-screening</t>
+  </si>
+  <si>
+    <t>2026-10-13T16:51:44.603Z</t>
+  </si>
+  <si>
+    <t>Cancer Screening | Find Care | PfizerForAll™</t>
+  </si>
+  <si>
+    <t>https://www.pfizerforall.com/find-care/cancer-screening/</t>
+  </si>
+  <si>
+    <t>find-care/prepare-for-care.report.json</t>
+  </si>
+  <si>
+    <t>["hero-page","cards-article","columns-media","cards-icon"]</t>
+  </si>
+  <si>
+    <t>find-care/prepare-for-care</t>
+  </si>
+  <si>
+    <t>2026-10-13T16:50:58.686Z</t>
+  </si>
+  <si>
+    <t>Prepare for Care | Find Care | PfizerForAll™</t>
+  </si>
+  <si>
+    <t>https://www.pfizerforall.com/find-care/prepare-for-care</t>
+  </si>
+  <si>
+    <t>find-care/talk-to-a-doctor.report.json</t>
+  </si>
+  <si>
+    <t>["hero-page","columns-media","cards-action"]</t>
+  </si>
+  <si>
+    <t>find-care/talk-to-a-doctor</t>
+  </si>
+  <si>
+    <t>2026-10-13T16:51:04.309Z</t>
+  </si>
+  <si>
+    <t>Talk to a Doctor | Find Care | PfizerForAll™</t>
+  </si>
+  <si>
+    <t>https://www.pfizerforall.com/find-care/talk-to-a-doctor</t>
+  </si>
+  <si>
+    <t>savings-support/prescription-assistance.report.json</t>
+  </si>
+  <si>
+    <t>["hero-page","cards-fact","columns-media","accordion-faq","search-prompt"]</t>
+  </si>
+  <si>
+    <t>savings-support/prescription-assistance</t>
+  </si>
+  <si>
+    <t>savings-support</t>
+  </si>
+  <si>
+    <t>2026-10-13T16:52:05.718Z</t>
+  </si>
+  <si>
+    <t>Prescription Assistance | PfizerForAll™</t>
+  </si>
+  <si>
+    <t>https://www.pfizerforall.com/savings-support/prescription-assistance</t>
+  </si>
+  <si>
+    <t>savings-support/self-pay.report.json</t>
+  </si>
+  <si>
+    <t>["hero-page","accordion-faq","search-prompt","cards-icon"]</t>
+  </si>
+  <si>
+    <t>savings-support/self-pay</t>
+  </si>
+  <si>
+    <t>2026-10-13T16:51:10.186Z</t>
+  </si>
+  <si>
+    <t>Self-Pay | PfizerForAll™</t>
+  </si>
+  <si>
+    <t>https://www.pfizerforall.com/savings-support/self-pay</t>
+  </si>
+  <si>
+    <t>fragments/find-care/cancer-screening/schedule-breast-screening.report.json</t>
+  </si>
+  <si>
+    <t>[]</t>
+  </si>
+  <si>
+    <t>fragments/find-care/cancer-screening/schedule-breast-screening</t>
+  </si>
+  <si>
+    <t>cancer-screening-fragment</t>
+  </si>
+  <si>
+    <t>2026-10-13T16:51:52.194Z</t>
+  </si>
+  <si>
+    <t>Fragment: schedule-breast-screening</t>
+  </si>
+  <si>
+    <t>https://www.pfizerforall.com/find-care/cancer-screening/#schedule-breast-screening</t>
+  </si>
+  <si>
+    <t>fragments/find-care/cancer-screening/schedule-cervical-screening.report.json</t>
+  </si>
+  <si>
+    <t>fragments/find-care/cancer-screening/schedule-cervical-screening</t>
+  </si>
+  <si>
+    <t>2026-10-13T16:51:58.706Z</t>
+  </si>
+  <si>
+    <t>Fragment: schedule-cervical-screening</t>
+  </si>
+  <si>
+    <t>https://www.pfizerforall.com/find-care/cancer-screening/#schedule-cervical-screening</t>
   </si>
 </sst>
 </file>
@@ -447,18 +663,16 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:H2"/>
+  <dimension ref="A1:I13"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
-    <col min="1" max="1" width="19" customWidth="1"/>
-    <col min="2" max="2" width="50" customWidth="1"/>
-    <col min="3" max="3" width="7" customWidth="1"/>
-    <col min="5" max="5" width="10" customWidth="1"/>
-    <col min="6" max="6" width="26" customWidth="1"/>
-    <col min="7" max="8" width="31" customWidth="1"/>
+    <col min="1" max="4" width="50" customWidth="1"/>
+    <col min="6" max="6" width="27" customWidth="1"/>
+    <col min="7" max="7" width="26" customWidth="1"/>
+    <col min="8" max="9" width="50" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" s="1" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:9" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -483,35 +697,360 @@
       <c r="H1" s="1" t="s">
         <v>7</v>
       </c>
-    </row>
-    <row r="2" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="I1" s="1" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="2" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="B2" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="C2" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="D2" t="s">
+        <v>12</v>
+      </c>
+      <c r="E2" t="s">
+        <v>13</v>
+      </c>
+      <c r="F2" t="s">
+        <v>14</v>
+      </c>
+      <c r="G2" t="s">
+        <v>15</v>
+      </c>
+      <c r="H2" t="s">
+        <v>16</v>
+      </c>
+      <c r="I2" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="3" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>18</v>
+      </c>
+      <c r="B3" t="s">
+        <v>19</v>
+      </c>
+      <c r="C3" t="s">
         <v>11</v>
       </c>
-      <c r="E2" t="s">
-        <v>12</v>
-      </c>
-      <c r="F2" t="s">
-        <v>13</v>
-      </c>
-      <c r="G2" t="s">
+      <c r="D3" t="s">
+        <v>20</v>
+      </c>
+      <c r="E3" t="s">
+        <v>13</v>
+      </c>
+      <c r="F3" t="s">
+        <v>20</v>
+      </c>
+      <c r="G3" t="s">
+        <v>21</v>
+      </c>
+      <c r="H3" t="s">
+        <v>22</v>
+      </c>
+      <c r="I3" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="4" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>24</v>
+      </c>
+      <c r="B4" t="s">
+        <v>25</v>
+      </c>
+      <c r="C4" t="s">
+        <v>11</v>
+      </c>
+      <c r="D4" t="s">
+        <v>26</v>
+      </c>
+      <c r="E4" t="s">
+        <v>13</v>
+      </c>
+      <c r="F4" t="s">
+        <v>27</v>
+      </c>
+      <c r="G4" t="s">
+        <v>28</v>
+      </c>
+      <c r="H4" t="s">
+        <v>29</v>
+      </c>
+      <c r="I4" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="5" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>31</v>
+      </c>
+      <c r="B5" t="s">
+        <v>32</v>
+      </c>
+      <c r="C5" t="s">
+        <v>11</v>
+      </c>
+      <c r="D5" t="s">
+        <v>33</v>
+      </c>
+      <c r="E5" t="s">
+        <v>13</v>
+      </c>
+      <c r="F5" t="s">
         <v>14</v>
       </c>
-      <c r="H2" t="s">
-        <v>15</v>
+      <c r="G5" t="s">
+        <v>34</v>
+      </c>
+      <c r="H5" t="s">
+        <v>35</v>
+      </c>
+      <c r="I5" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="6" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>37</v>
+      </c>
+      <c r="B6" t="s">
+        <v>38</v>
+      </c>
+      <c r="C6" t="s">
+        <v>11</v>
+      </c>
+      <c r="D6" t="s">
+        <v>39</v>
+      </c>
+      <c r="E6" t="s">
+        <v>13</v>
+      </c>
+      <c r="F6" t="s">
+        <v>14</v>
+      </c>
+      <c r="G6" t="s">
+        <v>40</v>
+      </c>
+      <c r="H6" t="s">
+        <v>41</v>
+      </c>
+      <c r="I6" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="7" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>43</v>
+      </c>
+      <c r="B7" t="s">
+        <v>44</v>
+      </c>
+      <c r="C7" t="s">
+        <v>45</v>
+      </c>
+      <c r="D7" t="s">
+        <v>46</v>
+      </c>
+      <c r="E7" t="s">
+        <v>13</v>
+      </c>
+      <c r="F7" t="s">
+        <v>47</v>
+      </c>
+      <c r="G7" t="s">
+        <v>48</v>
+      </c>
+      <c r="H7" t="s">
+        <v>49</v>
+      </c>
+      <c r="I7" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="8" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>51</v>
+      </c>
+      <c r="B8" t="s">
+        <v>52</v>
+      </c>
+      <c r="C8" t="s">
+        <v>11</v>
+      </c>
+      <c r="D8" t="s">
+        <v>53</v>
+      </c>
+      <c r="E8" t="s">
+        <v>13</v>
+      </c>
+      <c r="F8" t="s">
+        <v>14</v>
+      </c>
+      <c r="G8" t="s">
+        <v>54</v>
+      </c>
+      <c r="H8" t="s">
+        <v>55</v>
+      </c>
+      <c r="I8" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="9" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
+        <v>57</v>
+      </c>
+      <c r="B9" t="s">
+        <v>58</v>
+      </c>
+      <c r="C9" t="s">
+        <v>11</v>
+      </c>
+      <c r="D9" t="s">
+        <v>59</v>
+      </c>
+      <c r="E9" t="s">
+        <v>13</v>
+      </c>
+      <c r="F9" t="s">
+        <v>14</v>
+      </c>
+      <c r="G9" t="s">
+        <v>60</v>
+      </c>
+      <c r="H9" t="s">
+        <v>61</v>
+      </c>
+      <c r="I9" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="10" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
+        <v>63</v>
+      </c>
+      <c r="B10" t="s">
+        <v>64</v>
+      </c>
+      <c r="C10" t="s">
+        <v>11</v>
+      </c>
+      <c r="D10" t="s">
+        <v>65</v>
+      </c>
+      <c r="E10" t="s">
+        <v>13</v>
+      </c>
+      <c r="F10" t="s">
+        <v>66</v>
+      </c>
+      <c r="G10" t="s">
+        <v>67</v>
+      </c>
+      <c r="H10" t="s">
+        <v>68</v>
+      </c>
+      <c r="I10" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="11" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A11" t="s">
+        <v>70</v>
+      </c>
+      <c r="B11" t="s">
+        <v>71</v>
+      </c>
+      <c r="C11" t="s">
+        <v>11</v>
+      </c>
+      <c r="D11" t="s">
+        <v>72</v>
+      </c>
+      <c r="E11" t="s">
+        <v>13</v>
+      </c>
+      <c r="F11" t="s">
+        <v>14</v>
+      </c>
+      <c r="G11" t="s">
+        <v>73</v>
+      </c>
+      <c r="H11" t="s">
+        <v>74</v>
+      </c>
+      <c r="I11" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="12" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A12" t="s">
+        <v>76</v>
+      </c>
+      <c r="B12" t="s">
+        <v>77</v>
+      </c>
+      <c r="C12" t="s">
+        <v>11</v>
+      </c>
+      <c r="D12" t="s">
+        <v>78</v>
+      </c>
+      <c r="E12" t="s">
+        <v>13</v>
+      </c>
+      <c r="F12" t="s">
+        <v>79</v>
+      </c>
+      <c r="G12" t="s">
+        <v>80</v>
+      </c>
+      <c r="H12" t="s">
+        <v>81</v>
+      </c>
+      <c r="I12" t="s">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="13" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A13" t="s">
+        <v>83</v>
+      </c>
+      <c r="B13" t="s">
+        <v>77</v>
+      </c>
+      <c r="C13" t="s">
+        <v>11</v>
+      </c>
+      <c r="D13" t="s">
+        <v>84</v>
+      </c>
+      <c r="E13" t="s">
+        <v>13</v>
+      </c>
+      <c r="F13" t="s">
+        <v>79</v>
+      </c>
+      <c r="G13" t="s">
+        <v>85</v>
+      </c>
+      <c r="H13" t="s">
+        <v>86</v>
+      </c>
+      <c r="I13" t="s">
+        <v>87</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:H1"/>
+  <autoFilter ref="A1:I1"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
 </worksheet>

</xml_diff>